<commit_message>
modifiqué el archivo de pen sales para que hubiesen mas meses de diferencia entre las fechas y asi poder crear el diagrama de linea
</commit_message>
<xml_diff>
--- a/Data/Pen Sales Data.xlsx
+++ b/Data/Pen Sales Data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alice/Desktop/Course_Materials/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unanmanagua-my.sharepoint.com/personal/rene_sandoval23908226_estu_unan_edu_ni/Documents/UNAN 2023-2027/V Semestre/Analisis exploratorio de datos/Python 2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF10E04D-C46A-CB42-950C-0B504C1B54A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{CF10E04D-C46A-CB42-950C-0B504C1B54A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCEB44FD-0381-4C71-9678-D319373A8D7C}"/>
   <bookViews>
-    <workbookView xWindow="740" yWindow="500" windowWidth="28040" windowHeight="16000" xr2:uid="{88CB5200-0D19-2446-86AC-C4FBD1C615F9}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19406" windowHeight="11486" xr2:uid="{88CB5200-0D19-2446-86AC-C4FBD1C615F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Pen Sales" sheetId="1" r:id="rId1"/>
     <sheet name="Pen Costs" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,9 +24,10 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -161,8 +162,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -214,12 +215,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -539,19 +540,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B65F30A-E2C2-D84E-BD5E-139BBF0CA3F0}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="155.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="155.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -574,7 +575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>5201</v>
       </c>
@@ -597,7 +598,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3">
         <f>A2+1</f>
         <v>5202</v>
@@ -621,7 +622,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="0">A3+1</f>
         <v>5203</v>
@@ -645,7 +646,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>5204</v>
@@ -669,7 +670,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5205</v>
@@ -693,7 +694,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5206</v>
@@ -717,7 +718,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>5207</v>
@@ -741,7 +742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>5208</v>
@@ -765,7 +766,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>5209</v>
@@ -789,7 +790,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>5210</v>
@@ -813,7 +814,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>5211</v>
@@ -837,7 +838,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>5212</v>
@@ -861,7 +862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>5213</v>
@@ -885,7 +886,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>5214</v>
@@ -909,7 +910,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>5215</v>
@@ -933,7 +934,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>5216</v>
@@ -957,7 +958,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>5217</v>
@@ -981,7 +982,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>5218</v>
@@ -1005,7 +1006,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>5219</v>
@@ -1029,7 +1030,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>5220</v>
@@ -1053,7 +1054,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>5221</v>
@@ -1077,7 +1078,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>5222</v>
@@ -1101,7 +1102,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>5223</v>
@@ -1125,7 +1126,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>5224</v>
@@ -1149,7 +1150,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>5225</v>
@@ -1181,13 +1182,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{510D3640-C683-3941-B5B2-3C78F5934425}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.35546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>13</v>
       </c>
@@ -1195,7 +1196,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1203,7 +1204,7 @@
         <v>5.99</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1211,7 +1212,7 @@
         <v>12.99</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1219,7 +1220,7 @@
         <v>6.95</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>5.99</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1235,7 +1236,7 @@
         <v>12.99</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1432,13 +1433,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD506EFA-CF68-4EB5-A8AA-F6E42D705E41}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD506EFA-CF68-4EB5-A8AA-F6E42D705E41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1bb583d6-7de5-4467-bb06-9aeb8738f185"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7F82D2F-E708-4223-A587-34EE88DDC2ED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7F82D2F-E708-4223-A587-34EE88DDC2ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DF9CF85-D68B-497D-B89F-259FC52725F2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DF9CF85-D68B-497D-B89F-259FC52725F2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>